<commit_message>
Integrate soil aggregate data and update analyses
Added and processed new soil aggregate stability data, including merging datasets and calculating seasonal means. Updated ecological and economic synthesis scripts to incorporate aggregate stability, standardized values, and revised model specifications. Improved plots, added supplementary analyses, and updated documentation and todos to reflect new data integration and analysis steps.
</commit_message>
<xml_diff>
--- a/Data Analysis/1_Data/Aggregates/WSA_August_clean.xlsx
+++ b/Data Analysis/1_Data/Aggregates/WSA_August_clean.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aw52udov\Desktop\Masterarbeit\02_Methoden\03_WSA\01_RawData\02_August\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mm68tulo\Desktop\Jena Chapter\Data Analysis\1_Data\Aggregates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2432E190-B8A1-4041-8FA5-AE7A5B26D8AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DA1098-A808-4D6F-A688-EB6223F6B143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50" yWindow="0" windowWidth="19150" windowHeight="10540" xr2:uid="{BC0CCBAF-3D64-42AA-9871-21EBB1E9EF22}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BC0CCBAF-3D64-42AA-9871-21EBB1E9EF22}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,9 +36,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
   <si>
-    <t>Plot/Subplot/Site</t>
-  </si>
-  <si>
     <t>B1A01</t>
   </si>
   <si>
@@ -300,13 +297,16 @@
     <t>B4A15</t>
   </si>
   <si>
-    <t>Mean_Overall_Aggregates</t>
-  </si>
-  <si>
     <t>Mean_WSA</t>
   </si>
   <si>
     <t>WSA_sd</t>
+  </si>
+  <si>
+    <t>Plotcode</t>
+  </si>
+  <si>
+    <t>agg_overall</t>
   </si>
 </sst>
 </file>
@@ -414,7 +414,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -430,7 +430,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -727,46 +727,46 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28A87A7C-19B7-4DE5-8CAA-97D17BD78A89}">
   <dimension ref="A1:K96"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
       </c>
       <c r="B2" s="6">
         <v>90.250507786053134</v>
@@ -802,9 +802,9 @@
         <v>1.2701901924611934</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="6">
         <v>92.028469750889641</v>
@@ -840,9 +840,9 @@
         <v>1.0381973565105564</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="6">
         <v>84.236453201970448</v>
@@ -878,9 +878,9 @@
         <v>0.79907301965800992</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="6">
         <v>82.125930941096783</v>
@@ -916,9 +916,9 @@
         <v>1.835087304949754</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="6">
         <v>85.45454545454561</v>
@@ -954,9 +954,9 @@
         <v>1.1384799022590375</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="6">
         <v>93.535353535353323</v>
@@ -992,9 +992,9 @@
         <v>1.2729181674261698</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="6">
         <v>83.47768154563677</v>
@@ -1030,9 +1030,9 @@
         <v>1.4491106364799047</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="6">
         <v>83.873290136789009</v>
@@ -1068,9 +1068,9 @@
         <v>1.2226612839334923</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="6">
         <v>93.285990961910429</v>
@@ -1106,9 +1106,9 @@
         <v>0.60574372164681534</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="6">
         <v>87.8871300757054</v>
@@ -1144,9 +1144,9 @@
         <v>1.7984324548814026</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="6">
         <v>78.776713338246282</v>
@@ -1182,9 +1182,9 @@
         <v>0.61676776783198028</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="6">
         <v>94.034302759135258</v>
@@ -1220,9 +1220,9 @@
         <v>0.47523013390891272</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="6">
         <v>75.472928897586428</v>
@@ -1258,9 +1258,9 @@
         <v>0.28547950046162279</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="6">
         <v>90.841750841751406</v>
@@ -1296,9 +1296,9 @@
         <v>0.26287295169936814</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="6">
         <v>84.9966510381782</v>
@@ -1334,9 +1334,9 @@
         <v>3.0220288937591047</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="6">
         <v>84.996651038178086</v>
@@ -1372,9 +1372,9 @@
         <v>2.4186852943866888</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="6">
         <v>95.619438740588748</v>
@@ -1410,9 +1410,9 @@
         <v>2.5672225662061652</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="6">
         <v>95.690235690235795</v>
@@ -1448,9 +1448,9 @@
         <v>1.1041345927539703</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="6">
         <v>82.778864970645827</v>
@@ -1486,9 +1486,9 @@
         <v>0.77801030850428532</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="6">
         <v>96.34703196347067</v>
@@ -1524,9 +1524,9 @@
         <v>0.21819567027166478</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="6">
         <v>91.238877481177482</v>
@@ -1562,9 +1562,9 @@
         <v>1.2487542607991693</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="6">
         <v>91.831177671886081</v>
@@ -1600,9 +1600,9 @@
         <v>1.6470206276659853</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" s="6">
         <v>95.758780649436829</v>
@@ -1638,9 +1638,9 @@
         <v>0.68858382912889771</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="6">
         <v>79.961464354528005</v>
@@ -1676,9 +1676,9 @@
         <v>4.5264406957821475</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="6">
         <v>80.063897763578254</v>
@@ -1714,9 +1714,9 @@
         <v>0.59742618539854986</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="6">
         <v>93.455003146633345</v>
@@ -1752,9 +1752,9 @@
         <v>1.0062355031710066</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="6">
         <v>87.000677048069932</v>
@@ -1790,9 +1790,9 @@
         <v>1.1487613869714488</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="6">
         <v>92.996632996632499</v>
@@ -1828,9 +1828,9 @@
         <v>0.17950863284060337</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="6">
         <v>93.144363876071424</v>
@@ -1866,9 +1866,9 @@
         <v>0.20125729612001889</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" s="6">
         <v>94.612794612794175</v>
@@ -1904,9 +1904,9 @@
         <v>0.76743109794340525</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32" s="6">
         <v>91.092553931802499</v>
@@ -1942,9 +1942,9 @@
         <v>0.53481252444696969</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="6">
         <v>93.737769080234628</v>
@@ -1980,9 +1980,9 @@
         <v>0.8479972688146411</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="6">
         <v>86.571981923822221</v>
@@ -2018,9 +2018,9 @@
         <v>1.9139027241174604</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" s="6">
         <v>90.891840607210327</v>
@@ -2056,9 +2056,9 @@
         <v>0.69832252675083706</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" s="6">
         <v>93.167259786477359</v>
@@ -2094,9 +2094,9 @@
         <v>0.78338725021032574</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" s="6">
         <v>94.754098360656045</v>
@@ -2132,9 +2132,9 @@
         <v>0.7575910366497145</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B38" s="6">
         <v>84.233947870311425</v>
@@ -2170,9 +2170,9 @@
         <v>1.5498013873701348</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" s="6">
         <v>90.640055058499556</v>
@@ -2208,9 +2208,9 @@
         <v>0.70879919169927286</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B40" s="6">
         <v>93.319415448851544</v>
@@ -2246,9 +2246,9 @@
         <v>0.46774177464747024</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B41" s="6">
         <v>97.349237905898107</v>
@@ -2284,9 +2284,9 @@
         <v>0.70377074338392986</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="6">
         <v>91.092553931802584</v>
@@ -2322,9 +2322,9 @@
         <v>0.71789571199760172</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="6">
         <v>83.632982021078234</v>
@@ -2360,9 +2360,9 @@
         <v>0.59604595107052794</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B44" s="6">
         <v>84.819734345351165</v>
@@ -2398,9 +2398,9 @@
         <v>0.91254357814993559</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B45" s="6">
         <v>95.15151515151571</v>
@@ -2436,9 +2436,9 @@
         <v>0.87095194782219709</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" s="6">
         <v>94.28942245295265</v>
@@ -2474,9 +2474,9 @@
         <v>0.76943588462248369</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" s="6">
         <v>86.746189529489783</v>
@@ -2512,9 +2512,9 @@
         <v>2.8848609431580106</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B48" s="6">
         <v>95.228628230616138</v>
@@ -2550,9 +2550,9 @@
         <v>0.4196936048633933</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B49" s="6">
         <v>79.753406878650196</v>
@@ -2588,9 +2588,9 @@
         <v>1.3213915536096834</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B50" s="6">
         <v>97.912589693412016</v>
@@ -2626,9 +2626,9 @@
         <v>0.70234074579077554</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B51" s="6">
         <v>97.87939032471877</v>
@@ -2664,9 +2664,9 @@
         <v>0.67040940782783198</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B52" s="6">
         <v>90.535838552539943</v>
@@ -2702,9 +2702,9 @@
         <v>1.0765311142364291</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B53" s="6">
         <v>94.554118447924054</v>
@@ -2740,9 +2740,9 @@
         <v>0.26784852860922642</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B54" s="6">
         <v>93.282015395381123</v>
@@ -2778,9 +2778,9 @@
         <v>1.0568208224689581</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" s="6">
         <v>86.216037110669092</v>
@@ -2816,9 +2816,9 @@
         <v>1.2853994539498159</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B56" s="6">
         <v>81.639344262294799</v>
@@ -2854,9 +2854,9 @@
         <v>1.4522099028164248</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B57" s="6">
         <v>87.542315504401273</v>
@@ -2892,9 +2892,9 @@
         <v>0.72362659581047328</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B58" s="6">
         <v>95.071868583162043</v>
@@ -2930,9 +2930,9 @@
         <v>0.84592229268229613</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B59" s="6">
         <v>87.609427609427442</v>
@@ -2968,9 +2968,9 @@
         <v>1.1058850362708288</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B60" s="6">
         <v>97.785467128028102</v>
@@ -3006,9 +3006,9 @@
         <v>0.78097882269073937</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B61" s="6">
         <v>96.10299234516313</v>
@@ -3044,9 +3044,9 @@
         <v>0.42095657616378751</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A62" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B62" s="6">
         <v>97.833446174678059</v>
@@ -3082,9 +3082,9 @@
         <v>0.41031271022425986</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B63" s="6">
         <v>97.231833910034752</v>
@@ -3120,9 +3120,9 @@
         <v>0.69823990436771455</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B64" s="6">
         <v>96.036801132342902</v>
@@ -3158,9 +3158,9 @@
         <v>0.70824174810113683</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" s="6">
         <v>96.802131912059238</v>
@@ -3196,9 +3196,9 @@
         <v>0.64060145118089007</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B66" s="6">
         <v>90.792146242383126</v>
@@ -3234,9 +3234,9 @@
         <v>1.3528111269605725</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B67" s="6">
         <v>86.604152712659058</v>
@@ -3272,9 +3272,9 @@
         <v>1.2531893084066428</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B68" s="6">
         <v>94.137241838774187</v>
@@ -3310,9 +3310,9 @@
         <v>0.79101800262462163</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B69" s="6">
         <v>57.811470006592067</v>
@@ -3348,9 +3348,9 @@
         <v>2.5359479369864997</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B70" s="6">
         <v>96.948506039415008</v>
@@ -3386,9 +3386,9 @@
         <v>0.38765901619644999</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B71" s="6">
         <v>89.167230873391873</v>
@@ -3424,9 +3424,9 @@
         <v>2.1163639124820137</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B72" s="6">
         <v>68.332251784555496</v>
@@ -3462,9 +3462,9 @@
         <v>1.614574712269129</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B73" s="6">
         <v>67.64514024787988</v>
@@ -3500,9 +3500,9 @@
         <v>2.2455387917816254</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B74" s="6">
         <v>84.625579854207814</v>
@@ -3538,9 +3538,9 @@
         <v>1.9090034081531242</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B75" s="6">
         <v>88.866799204770999</v>
@@ -3576,9 +3576,9 @@
         <v>1.1814073601256498</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B76" s="6">
         <v>84.344422700587188</v>
@@ -3614,9 +3614,9 @@
         <v>0.98658278767594187</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B77" s="6">
         <v>76.918032786884822</v>
@@ -3652,9 +3652,9 @@
         <v>2.4889137199505376</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B78" s="6">
         <v>93.354632587859655</v>
@@ -3690,9 +3690,9 @@
         <v>2.776941794086774</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B79" s="6">
         <v>76.324845147969341</v>
@@ -3728,9 +3728,9 @@
         <v>3.3403579007038156</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B80" s="6">
         <v>78.420038535645332</v>
@@ -3766,9 +3766,9 @@
         <v>0.79601436744937093</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B81" s="6">
         <v>91.44115796098167</v>
@@ -3804,63 +3804,63 @@
         <v>14.153227890531626</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="J82" s="6"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="J83" s="6"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="J84" s="6"/>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
       <c r="J85" s="6"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
       <c r="J86" s="6"/>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="J87" s="6"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
       <c r="J88" s="6"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="J89" s="6"/>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="J90" s="6"/>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="J91" s="6"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="J92" s="6"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="J93" s="6"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
       <c r="J94" s="6"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="J95" s="6"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="J96" s="6"/>
     </row>

</xml_diff>